<commit_message>
Add dynamic user input for any stock ticker
</commit_message>
<xml_diff>
--- a/stock_analysis.xlsx
+++ b/stock_analysis.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -490,19 +490,19 @@
         <v>379.29</v>
       </c>
       <c r="D2" t="n">
-        <v>368.92</v>
+        <v>369.27</v>
       </c>
       <c r="E2" t="n">
-        <v>-2.73</v>
+        <v>-2.64</v>
       </c>
       <c r="F2" t="n">
         <v>1.67</v>
       </c>
       <c r="G2" t="n">
-        <v>404.62</v>
+        <v>404.63</v>
       </c>
       <c r="H2" t="n">
-        <v>475.77</v>
+        <v>475.78</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -525,10 +525,10 @@
         <v>222.22</v>
       </c>
       <c r="D3" t="n">
-        <v>254.36</v>
+        <v>254.68</v>
       </c>
       <c r="E3" t="n">
-        <v>14.46</v>
+        <v>14.61</v>
       </c>
       <c r="F3" t="n">
         <v>1.99</v>
@@ -548,278 +548,103 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Wells Fargo</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>WFC</t>
+          <t>GOOG</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>69.79000000000001</v>
+        <v>158.33</v>
       </c>
       <c r="D4" t="n">
-        <v>80.73</v>
+        <v>295.11</v>
       </c>
       <c r="E4" t="n">
-        <v>15.67</v>
+        <v>86.38</v>
       </c>
       <c r="F4" t="n">
-        <v>1.85</v>
+        <v>1.9</v>
       </c>
       <c r="G4" t="n">
-        <v>83.98999999999999</v>
+        <v>310.72</v>
       </c>
       <c r="H4" t="n">
-        <v>83.54000000000001</v>
+        <v>264.58</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>HOLD</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>JPMorgan Chase</t>
+          <t>Goldman Sachs</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>JPM</t>
+          <t>GS</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>238.76</v>
+        <v>537.3200000000001</v>
       </c>
       <c r="D5" t="n">
-        <v>294.52</v>
+        <v>858.73</v>
       </c>
       <c r="E5" t="n">
-        <v>23.35</v>
+        <v>59.82</v>
       </c>
       <c r="F5" t="n">
-        <v>1.59</v>
+        <v>2.03</v>
       </c>
       <c r="G5" t="n">
-        <v>299.18</v>
+        <v>876.25</v>
       </c>
       <c r="H5" t="n">
-        <v>300.69</v>
+        <v>800.72</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>HOLD</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Oracle</t>
+          <t>Nvidia</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>140.52</v>
+        <v>110.12</v>
       </c>
       <c r="D6" t="n">
-        <v>144.9</v>
+        <v>175.54</v>
       </c>
       <c r="E6" t="n">
-        <v>3.12</v>
+        <v>59.4</v>
       </c>
       <c r="F6" t="n">
-        <v>3.9</v>
+        <v>2.61</v>
       </c>
       <c r="G6" t="n">
-        <v>154.72</v>
+        <v>182.76</v>
       </c>
       <c r="H6" t="n">
-        <v>217.87</v>
+        <v>179.64</v>
       </c>
       <c r="I6" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Google</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>GOOG</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>158.33</v>
-      </c>
-      <c r="D7" t="n">
-        <v>294.31</v>
-      </c>
-      <c r="E7" t="n">
-        <v>85.88</v>
-      </c>
-      <c r="F7" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="G7" t="n">
-        <v>310.7</v>
-      </c>
-      <c r="H7" t="n">
-        <v>264.57</v>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Nvidia</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>NVDA</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>110.12</v>
-      </c>
-      <c r="D8" t="n">
-        <v>175.33</v>
-      </c>
-      <c r="E8" t="n">
-        <v>59.21</v>
-      </c>
-      <c r="F8" t="n">
-        <v>2.61</v>
-      </c>
-      <c r="G8" t="n">
-        <v>182.75</v>
-      </c>
-      <c r="H8" t="n">
-        <v>179.63</v>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>AMZN</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>192.17</v>
-      </c>
-      <c r="D9" t="n">
-        <v>210.05</v>
-      </c>
-      <c r="E9" t="n">
-        <v>9.300000000000001</v>
-      </c>
-      <c r="F9" t="n">
-        <v>2.21</v>
-      </c>
-      <c r="G9" t="n">
-        <v>215.42</v>
-      </c>
-      <c r="H9" t="n">
-        <v>224.58</v>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>SELL</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Goldman Sachs</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>GS</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>537.3200000000001</v>
-      </c>
-      <c r="D10" t="n">
-        <v>858.62</v>
-      </c>
-      <c r="E10" t="n">
-        <v>59.8</v>
-      </c>
-      <c r="F10" t="n">
-        <v>2.03</v>
-      </c>
-      <c r="G10" t="n">
-        <v>876.25</v>
-      </c>
-      <c r="H10" t="n">
-        <v>800.72</v>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Boeing</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>BA</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>168.17</v>
-      </c>
-      <c r="D11" t="n">
-        <v>207.31</v>
-      </c>
-      <c r="E11" t="n">
-        <v>23.27</v>
-      </c>
-      <c r="F11" t="n">
-        <v>2.33</v>
-      </c>
-      <c r="G11" t="n">
-        <v>225.02</v>
-      </c>
-      <c r="H11" t="n">
-        <v>218.58</v>
-      </c>
-      <c r="I11" t="inlineStr">
         <is>
           <t>SELL</t>
         </is>

</xml_diff>

<commit_message>
Add Apple DCF valuation model
</commit_message>
<xml_diff>
--- a/stock_analysis.xlsx
+++ b/stock_analysis.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,7 +478,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>microsoft</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -487,13 +487,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>379.29</v>
+        <v>379.24</v>
       </c>
       <c r="D2" t="n">
-        <v>369.27</v>
+        <v>369.37</v>
       </c>
       <c r="E2" t="n">
-        <v>-2.64</v>
+        <v>-2.6</v>
       </c>
       <c r="F2" t="n">
         <v>1.67</v>
@@ -513,140 +513,70 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>222.22</v>
+        <v>196.01</v>
       </c>
       <c r="D3" t="n">
-        <v>254.68</v>
+        <v>210.57</v>
       </c>
       <c r="E3" t="n">
-        <v>14.61</v>
+        <v>7.43</v>
       </c>
       <c r="F3" t="n">
-        <v>1.99</v>
+        <v>2.21</v>
       </c>
       <c r="G3" t="n">
-        <v>260.11</v>
+        <v>215.43</v>
       </c>
       <c r="H3" t="n">
-        <v>248.51</v>
+        <v>224.58</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>SELL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Cisco</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>158.33</v>
+        <v>60.35</v>
       </c>
       <c r="D4" t="n">
-        <v>295.11</v>
+        <v>77.93000000000001</v>
       </c>
       <c r="E4" t="n">
-        <v>86.38</v>
+        <v>29.12</v>
       </c>
       <c r="F4" t="n">
-        <v>1.9</v>
+        <v>1.77</v>
       </c>
       <c r="G4" t="n">
-        <v>310.72</v>
+        <v>79.12</v>
       </c>
       <c r="H4" t="n">
-        <v>264.58</v>
+        <v>72.75</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
           <t>HOLD</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Goldman Sachs</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>GS</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>537.3200000000001</v>
-      </c>
-      <c r="D5" t="n">
-        <v>858.73</v>
-      </c>
-      <c r="E5" t="n">
-        <v>59.82</v>
-      </c>
-      <c r="F5" t="n">
-        <v>2.03</v>
-      </c>
-      <c r="G5" t="n">
-        <v>876.25</v>
-      </c>
-      <c r="H5" t="n">
-        <v>800.72</v>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Nvidia</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>NVDA</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>110.12</v>
-      </c>
-      <c r="D6" t="n">
-        <v>175.54</v>
-      </c>
-      <c r="E6" t="n">
-        <v>59.4</v>
-      </c>
-      <c r="F6" t="n">
-        <v>2.61</v>
-      </c>
-      <c r="G6" t="n">
-        <v>182.76</v>
-      </c>
-      <c r="H6" t="n">
-        <v>179.64</v>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>SELL</t>
         </is>
       </c>
     </row>

</xml_diff>